<commit_message>
Add Composicao sheet (sapata/emenda), chumbador pending, confirm placa qty
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0161y9YT6s3qhV5Y18zQkN9x
</commit_message>
<xml_diff>
--- a/drive-in/catalogo/CATALOGO.xlsx
+++ b/drive-in/catalogo/CATALOGO.xlsx
@@ -9,25 +9,27 @@
   <sheets>
     <sheet name="LEIA-ME" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Produtos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Colunas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sapatas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Tala e fixadores" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Travessas" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Diagonais" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Placa niveladora" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Braços" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Outros" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Composição" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Colunas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Sapatas" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Tala e fixadores" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Travessas" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Diagonais" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Placa niveladora" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Braços" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Outros" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Produtos'!$A$1:$S$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Colunas'!$A$1:$E$514</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sapatas'!$A$1:$G$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tala e fixadores'!$A$1:$G$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Travessas'!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Diagonais'!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Placa niveladora'!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Braços'!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Outros'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Composição'!$A$1:$G$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Colunas'!$A$1:$E$514</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sapatas'!$A$1:$G$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Tala e fixadores'!$A$1:$G$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Travessas'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Diagonais'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Placa niveladora'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Braços'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Outros'!$A$1:$E$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -83,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -91,6 +93,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -490,7 +495,13 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>"Composição": o que entra em cada conjunto (sapata, emenda) e em que quantidade. Parafusos e chumbadores ficam aqui, ligados ao item em "Produtos".</t>
+        </is>
+      </c>
+    </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -555,6 +566,55 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
+          <t>Coluna</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Vão (mm)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
           <t>Tipo</t>
         </is>
       </c>
@@ -586,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S30"/>
+  <dimension ref="A1:S32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -747,8 +807,6 @@
           <t>Civil 300</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>kg</t>
@@ -770,7 +828,6 @@
           <t>1 por coluna</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2" s="3" t="inlineStr">
         <is>
           <t>SEM CÓDIGO</t>
@@ -826,8 +883,6 @@
           <t>Civil 300</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>kg</t>
@@ -849,13 +904,11 @@
           <t>1 por coluna</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -901,8 +954,6 @@
           <t>Civil 300</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>kg</t>
@@ -924,13 +975,11 @@
           <t>1 por coluna</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -957,11 +1006,6 @@
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>kg</t>
@@ -975,13 +1019,11 @@
           <t>planilha</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
           <t>1 por coluna</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
       <c r="R5" s="3" t="inlineStr">
         <is>
           <t>SEM CÓDIGO</t>
@@ -1029,7 +1071,6 @@
           <t>0004.0003.03.001</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>Civil 300</t>
@@ -1048,15 +1089,11 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
           <t>1 por sapata</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1092,13 +1129,11 @@
           <t>SA</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>0004.0003.03.002</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>Civil 300</t>
@@ -1107,27 +1142,21 @@
       <c r="J7" t="n">
         <v>2.65</v>
       </c>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
           <t>1 por sapata</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr"/>
       <c r="R7" s="3" t="inlineStr">
         <is>
           <t>SEM CÓDIGO</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1163,7 +1192,6 @@
           <t>0004.0003.03.002</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>Civil 300</t>
@@ -1172,21 +1200,16 @@
       <c r="J8" t="n">
         <v>2.65</v>
       </c>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
           <t>1 por sapata</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1232,7 +1255,6 @@
           <t>0004.0003.03.002</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>Civil 300</t>
@@ -1241,27 +1263,21 @@
       <c r="J9" t="n">
         <v>2.65</v>
       </c>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
           <t>1 por sapata</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1335,10 +1351,9 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2 por sapata (planilha) [confirmar]</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr"/>
+          <t>2 por sapata</t>
+        </is>
+      </c>
       <c r="R10" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1422,16 +1437,14 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2 por sapata (planilha) [confirmar]</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr"/>
+          <t>2 por sapata</t>
+        </is>
+      </c>
       <c r="R11" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1508,7 +1521,6 @@
           <t>2 por emenda</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1536,7 +1548,6 @@
           <t>Parafuso 5/16" x 3/4" UNC ZNB</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>INT</t>
@@ -1547,29 +1558,21 @@
           <t>INT0648</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
           <t>(sem peso)</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
           <t>16 por emenda</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1597,7 +1600,6 @@
           <t>Porca sextavada 5/16" zincada</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>INT</t>
@@ -1608,35 +1610,26 @@
           <t>INT0650</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
           <t>(sem peso)</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
           <t>16 por emenda</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1654,7 +1647,6 @@
           <t>Arruela lisa 5/16" 8,5x20x1,2 zinc. BRC</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>INT</t>
@@ -1665,35 +1657,26 @@
           <t>INT0812</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>(sem peso)</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
           <t>32 por emenda</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1724,8 +1707,6 @@
           <t>ver aba Colunas (por altura)</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>Civil 300</t>
@@ -1752,13 +1733,11 @@
           <t>calculado (sliter fechado, sem descontar furos)</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
           <t>por altura</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1799,8 +1778,6 @@
           <t>ver aba Colunas (por altura)</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>Civil 300</t>
@@ -1827,13 +1804,11 @@
           <t>calculado (sliter fechado, sem descontar furos)</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
           <t>por altura</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1874,8 +1849,6 @@
           <t>ver aba Colunas (por altura)</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
           <t>Civil 300</t>
@@ -1902,13 +1875,11 @@
           <t>calculado (sliter fechado, sem descontar furos)</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
           <t>por altura</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1949,8 +1920,6 @@
           <t>ver aba Colunas (por altura)</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>Civil 300</t>
@@ -1977,13 +1946,11 @@
           <t>calculado (sliter fechado, sem descontar furos)</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
           <t>por altura</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2024,8 +1991,6 @@
           <t>ver aba Colunas (por altura)</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>Civil 300</t>
@@ -2052,13 +2017,11 @@
           <t>calculado (sliter fechado, sem descontar furos)</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
           <t>por altura</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2099,8 +2062,6 @@
           <t>ver aba Colunas (por altura)</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>Civil 300</t>
@@ -2127,13 +2088,11 @@
           <t>calculado (sliter fechado, sem descontar furos)</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
           <t>por altura</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2174,8 +2133,6 @@
           <t>ver aba Colunas (por altura)</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>Civil 300</t>
@@ -2202,13 +2159,11 @@
           <t>calculado (sliter fechado, sem descontar furos)</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
           <t>por altura</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2249,8 +2204,6 @@
           <t>ver aba Colunas (por altura)</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>Civil 300</t>
@@ -2277,13 +2230,11 @@
           <t>calculado (sliter fechado, sem descontar furos)</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
           <t>por altura</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2324,8 +2275,6 @@
           <t>ver aba Colunas (por altura)</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>Civil 300</t>
@@ -2352,13 +2301,11 @@
           <t>calculado (sliter fechado, sem descontar furos)</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
           <t>por altura</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2399,8 +2346,6 @@
           <t>ver aba Colunas (por altura)</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>Civil 300</t>
@@ -2427,13 +2372,11 @@
           <t>calculado (sliter fechado, sem descontar furos)</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
           <t>por altura</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2474,8 +2417,6 @@
           <t>ver aba Colunas (por altura)</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
           <t>Civil 300</t>
@@ -2502,13 +2443,11 @@
           <t>calculado (sliter fechado, sem descontar furos)</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
           <t>por altura</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2549,8 +2488,6 @@
           <t>ver aba Colunas (por altura)</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
           <t>Civil 300</t>
@@ -2577,13 +2514,11 @@
           <t>calculado (sliter fechado, sem descontar furos)</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
           <t>por altura</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2624,8 +2559,6 @@
           <t>ver aba Colunas (por altura)</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
           <t>Civil 300</t>
@@ -2652,13 +2585,11 @@
           <t>calculado (sliter fechado, sem descontar furos)</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
           <t>por altura</t>
         </is>
       </c>
-      <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2699,8 +2630,6 @@
           <t>ver aba Colunas (por altura)</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>Civil 300</t>
@@ -2727,13 +2656,11 @@
           <t>calculado (sliter fechado, sem descontar furos)</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
           <t>por altura</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2774,8 +2701,6 @@
           <t>ver aba Colunas (por altura)</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>Civil 300</t>
@@ -2802,13 +2727,11 @@
           <t>calculado (sliter fechado, sem descontar furos)</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
         <is>
           <t>por altura</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2817,6 +2740,120 @@
       <c r="S30" t="inlineStr">
         <is>
           <t>Peso teórico: sliter x espessura x 7,85e-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>CHUMB</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Fixador</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Chumbador 3/8" x 3"</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>(sem peso)</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>por sapata (ver Composição)</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" s="3" t="inlineStr">
+        <is>
+          <t>SEM CÓDIGO</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Código INT e quantidade a confirmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>FIX-SAP</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Fixador</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Parafuso/porca/arruela de fixação sapata-coluna</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>(sem peso)</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>por sapata (ver Composição)</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" s="3" t="inlineStr">
+        <is>
+          <t>SEM CÓDIGO</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Quais INT e quantidades: a confirmar</t>
         </is>
       </c>
     </row>
@@ -2827,6 +2864,714 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Conjunto (pai)</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Item (ID em Produtos)</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Descrição do item</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Quantidade</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Contagem</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SAP-80</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SAP-BASE</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PP BASE SAPATA</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>por sapata</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>desenho 0004.0003.02.001</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SAP-80</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SAP-U80</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Perfil U sapata 80</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>por sapata</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SAP-80</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PLN-80-101</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Placa niveladora</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>por sapata</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>confirmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SAP-80</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CHUMB</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Chumbador 3/8" x 3"</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>por sapata</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>A CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>4 era o valor da planilha antiga; código INT pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SAP-80</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>FIX-SAP</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Fixação sapata-coluna</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>por sapata</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>A CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>definir itens INT e quantidades</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SAP-101</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SAP-BASE</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>PP BASE SAPATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>por sapata</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>desenho 0004.0003.02.001</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SAP-101</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SAP-U101</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Perfil U sapata 101</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>por sapata</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SAP-101</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PLN-80-101</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Placa niveladora</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>por sapata</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>confirmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SAP-101</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CHUMB</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Chumbador 3/8" x 3"</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>por sapata</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>A CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>4 era o valor da planilha antiga; código INT pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SAP-101</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>FIX-SAP</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Fixação sapata-coluna</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>por sapata</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>A CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>definir itens INT e quantidades</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SAP-122</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>SAP-BASE</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>PP BASE SAPATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>por sapata</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>desenho 0004.0003.02.001</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SAP-122</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>SAP-U122</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Perfil U sapata 122</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>por sapata</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SAP-122</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PLN-122</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Placa niveladora</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>por sapata</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>confirmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SAP-122</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CHUMB</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Chumbador 3/8" x 3"</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>por sapata</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>A CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>4 era o valor da planilha antiga; código INT pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SAP-122</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>FIX-SAP</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Fixação sapata-coluna</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>por sapata</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>A CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>definir itens INT e quantidades</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>EMENDA</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>TAL</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>PP EMENDA COLUNA (tala)</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>por emenda</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>metade em cada coluna; só acima de 8500 mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>EMENDA</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>INT0648</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Parafuso 5/16" x 3/4"</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>16</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>por emenda</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>8 por tala</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>EMENDA</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>INT0650</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Porca 5/16"</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>16</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>por emenda</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>8 por tala</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>EMENDA</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>INT0812</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Arruela lisa 5/16"</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>32</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>por emenda</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>16 por tala</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G20"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14362,7 +15107,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14657,7 +15402,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14797,55 +15542,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:G5"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Descrição</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Perfil coluna</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Comprimento (mm)</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Código</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:E1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14905,6 +15601,55 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Perfil coluna</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Comprimento (mm)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -15006,56 +15751,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:E1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Descrição</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Coluna</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Vão (mm)</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Código</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>

</xml_diff>

<commit_message>
Complete sapata composition: chumbador INT0654 and fixing hardware
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0161y9YT6s3qhV5Y18zQkN9x
</commit_message>
<xml_diff>
--- a/drive-in/catalogo/CATALOGO.xlsx
+++ b/drive-in/catalogo/CATALOGO.xlsx
@@ -21,7 +21,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Produtos'!$A$1:$S$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Composição'!$A$1:$G$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Composição'!$A$1:$G$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Colunas'!$A$1:$E$514</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sapatas'!$A$1:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Tala e fixadores'!$A$1:$G$5</definedName>
@@ -646,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S32"/>
+  <dimension ref="A1:S31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Planilha usava 0,225 kg; aqui o peso do desenho</t>
+          <t>Planilha usava 0,225 kg; aqui o peso do desenho Fica entre a sapata e o piso.</t>
         </is>
       </c>
     </row>
@@ -1445,6 +1445,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Fica entre a sapata e o piso.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1570,7 +1575,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>16 por emenda</t>
+          <t>ver Composição</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1580,7 +1585,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Custo entra na aba de custo</t>
+          <t>Usado na sapata e na emenda</t>
         </is>
       </c>
     </row>
@@ -1622,12 +1627,17 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>16 por emenda</t>
+          <t>ver Composição</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Usado na sapata e na emenda</t>
         </is>
       </c>
     </row>
@@ -1669,12 +1679,17 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>32 por emenda</t>
+          <t>ver Composição</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Usado na sapata e na emenda</t>
         </is>
       </c>
     </row>
@@ -2756,106 +2771,40 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Chumbador 3/8" x 3"</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr"/>
+          <t>Chumbador PBA 3/8" x 3.1/2"</t>
+        </is>
+      </c>
       <c r="E31" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>INT0654</t>
+        </is>
+      </c>
       <c r="L31" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr">
         <is>
           <t>(sem peso)</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
-          <t>por sapata (ver Composição)</t>
-        </is>
-      </c>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" s="3" t="inlineStr">
-        <is>
-          <t>SEM CÓDIGO</t>
-        </is>
-      </c>
-      <c r="S31" t="inlineStr">
-        <is>
-          <t>Código INT e quantidade a confirmar</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>FIX-SAP</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Fixador</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Parafuso/porca/arruela de fixação sapata-coluna</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>(sem peso)</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>por sapata (ver Composição)</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" s="3" t="inlineStr">
-        <is>
-          <t>SEM CÓDIGO</t>
-        </is>
-      </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>Quais INT e quantidades: a confirmar</t>
-        </is>
-      </c>
+          <t>ver Composição</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:S30"/>
@@ -2869,7 +2818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2877,7 +2826,7 @@
     <col width="42" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3015,7 +2964,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>confirmado</t>
+          <t>fica entre a sapata e o piso</t>
         </is>
       </c>
     </row>
@@ -3027,12 +2976,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CHUMB</t>
+          <t>INT0654</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Chumbador 3/8" x 3"</t>
+          <t>Chumbador PBA 3/8" x 3.1/2"</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -3043,14 +2992,14 @@
           <t>por sapata</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>A CONFIRMAR</t>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>4 era o valor da planilha antiga; código INT pendente</t>
+          <t>sempre 4</t>
         </is>
       </c>
     </row>
@@ -3062,49 +3011,51 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>FIX-SAP</t>
+          <t>INT0648</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fixação sapata-coluna</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr"/>
+          <t>Parafuso 5/16" x 3/4" UNC ZNB</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4</v>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>por sapata</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>A CONFIRMAR</t>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>definir itens INT e quantidades</t>
+          <t>fixação da sapata</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SAP-101</t>
+          <t>SAP-80</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SAP-BASE</t>
+          <t>INT0650</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PP BASE SAPATA</t>
+          <t>Porca sextavada 5/16" zincada</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -3118,28 +3069,28 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>desenho 0004.0003.02.001</t>
+          <t>fixação da sapata</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SAP-101</t>
+          <t>SAP-80</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SAP-U101</t>
+          <t>INT0812</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Perfil U sapata 101</t>
+          <t>Arruela lisa 5/16" 8,5x20x1,2</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -3151,7 +3102,11 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>fixação da sapata</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3161,16 +3116,16 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PLN-80-101</t>
+          <t>SAP-BASE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Placa niveladora</t>
+          <t>PP BASE SAPATA</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -3184,7 +3139,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>confirmado</t>
+          <t>desenho 0004.0003.02.001</t>
         </is>
       </c>
     </row>
@@ -3196,32 +3151,28 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CHUMB</t>
+          <t>SAP-U101</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Chumbador 3/8" x 3"</t>
+          <t>Perfil U sapata 101</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
           <t>por sapata</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>A CONFIRMAR</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>4 era o valor da planilha antiga; código INT pendente</t>
-        </is>
-      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3231,49 +3182,51 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>FIX-SAP</t>
+          <t>PLN-80-101</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fixação sapata-coluna</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr"/>
+          <t>Placa niveladora</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>por sapata</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>A CONFIRMAR</t>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>definir itens INT e quantidades</t>
+          <t>fica entre a sapata e o piso</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SAP-122</t>
+          <t>SAP-101</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SAP-BASE</t>
+          <t>INT0654</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>PP BASE SAPATA</t>
+          <t>Chumbador PBA 3/8" x 3.1/2"</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -3287,28 +3240,28 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>desenho 0004.0003.02.001</t>
+          <t>sempre 4</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SAP-122</t>
+          <t>SAP-101</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SAP-U122</t>
+          <t>INT0648</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Perfil U sapata 122</t>
+          <t>Parafuso 5/16" x 3/4" UNC ZNB</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -3320,26 +3273,30 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>fixação da sapata</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SAP-122</t>
+          <t>SAP-101</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PLN-122</t>
+          <t>INT0650</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Placa niveladora</t>
+          <t>Porca sextavada 5/16" zincada</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -3353,42 +3310,42 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>confirmado</t>
+          <t>fixação da sapata</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SAP-122</t>
+          <t>SAP-101</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CHUMB</t>
+          <t>INT0812</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Chumbador 3/8" x 3"</t>
+          <t>Arruela lisa 5/16" 8,5x20x1,2</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
           <t>por sapata</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>A CONFIRMAR</t>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4 era o valor da planilha antiga; código INT pendente</t>
+          <t>fixação da sapata</t>
         </is>
       </c>
     </row>
@@ -3400,53 +3357,55 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>FIX-SAP</t>
+          <t>SAP-BASE</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Fixação sapata-coluna</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr"/>
+          <t>PP BASE SAPATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
           <t>por sapata</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>A CONFIRMAR</t>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>definir itens INT e quantidades</t>
+          <t>desenho 0004.0003.02.001</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>EMENDA</t>
+          <t>SAP-122</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>TAL</t>
+          <t>SAP-U122</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PP EMENDA COLUNA (tala)</t>
+          <t>Perfil U sapata 122</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>por emenda</t>
+          <t>por sapata</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -3454,34 +3413,30 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>metade em cada coluna; só acima de 8500 mm</t>
-        </is>
-      </c>
+      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>EMENDA</t>
+          <t>SAP-122</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>INT0648</t>
+          <t>PLN-122</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Parafuso 5/16" x 3/4"</t>
+          <t>Placa niveladora</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>por emenda</t>
+          <t>por sapata</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -3491,32 +3446,32 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>8 por tala</t>
+          <t>fica entre a sapata e o piso</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>EMENDA</t>
+          <t>SAP-122</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>INT0650</t>
+          <t>INT0654</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Porca 5/16"</t>
+          <t>Chumbador PBA 3/8" x 3.1/2"</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>por emenda</t>
+          <t>por sapata</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -3526,47 +3481,257 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>8 por tala</t>
+          <t>sempre 4</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>SAP-122</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>INT0648</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Parafuso 5/16" x 3/4" UNC ZNB</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>por sapata</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>fixação da sapata</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SAP-122</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>INT0650</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Porca sextavada 5/16" zincada</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>4</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>por sapata</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>fixação da sapata</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SAP-122</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>INT0812</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Arruela lisa 5/16" 8,5x20x1,2</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>8</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>por sapata</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>fixação da sapata</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>EMENDA</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>TAL</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>PP EMENDA COLUNA (tala)</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>por emenda</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>metade em cada coluna; só acima de 8500 mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>EMENDA</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>INT0648</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Parafuso 5/16" x 3/4"</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>16</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>por emenda</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>8 por tala</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>EMENDA</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>INT0650</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Porca 5/16"</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>16</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>por emenda</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>8 por tala</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>EMENDA</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>INT0812</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Arruela lisa 5/16"</t>
         </is>
       </c>
-      <c r="D20" t="n">
+      <c r="D26" t="n">
         <v>32</v>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>por emenda</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
         <is>
           <t>16 por tala</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G20"/>
+  <autoFilter ref="A1:G26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15408,7 +15573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -15535,6 +15700,29 @@
         </is>
       </c>
       <c r="E5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Chumbador PBA 3/8" x 3.1/2"</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>INT0654</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>OK</t>
         </is>

</xml_diff>

<commit_message>
Add travessa/diagonal SA tables with checks; record confirmations
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0161y9YT6s3qhV5Y18zQkN9x
</commit_message>
<xml_diff>
--- a/drive-in/catalogo/CATALOGO.xlsx
+++ b/drive-in/catalogo/CATALOGO.xlsx
@@ -25,8 +25,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Colunas'!$A$1:$E$514</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sapatas'!$A$1:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Tala e fixadores'!$A$1:$G$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Travessas'!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Diagonais'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Travessas'!$A$1:$H$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Diagonais'!$A$1:$I$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Placa niveladora'!$A$1:$E$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Braços'!$A$1:$E$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Outros'!$A$1:$E$1</definedName>
@@ -505,14 +505,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Prefixos: SA = semiacabado | CO = composto/conjunto | INT = fixadores/itens INT (código da fábrica).</t>
+          <t>Itens sem código entram no BOM como "SAXXXX" (regra do responsável técnico).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Regra do app: código em branco (célula amarela) = item SEM CÓDIGO. O BOM mostra "SEM CÓDIGO" e o cálculo de peso segue normal.</t>
+          <t>Travessas/Diagonais: o app procura o SA pelo comprimento calculado, tolerância ±3 mm.</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S31"/>
+  <dimension ref="A1:S33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2804,7 +2804,168 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="S31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>TRAV-H</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Travessa horizontal</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Travessa horizontal (perfil)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>todas</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>ver aba Travessas</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>0004.0001.03.009</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>ACO0602 SLITER FF 1,40 x 80 GI</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>sliter 80; seção 30 x 22</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>kg/m</t>
+        </is>
+      </c>
+      <c r="M32" t="n">
+        <v>0.8792</v>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>calculado (sliter fechado)</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>por lateral (ver regras)</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Peso da tabela do SolidWorks não usado (inconsistente entre horizontal e diagonal). Comprimento total = A−78,6</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>TRAV-D</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Travessa diagonal</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Travessa diagonal (perfil)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>todas</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>ver aba Diagonais</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>0004.0001.03.009</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>ACO0602 SLITER FF 1,40 x 80 GI</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>sliter 80; seção 30 x 22</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>kg/m</t>
+        </is>
+      </c>
+      <c r="M33" t="n">
+        <v>0.8792</v>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>calculado (sliter fechado)</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>por vão entre horizontais</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Comprimento total = √(B²+V²)+30,5</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:S30"/>
@@ -2931,7 +3092,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3172,7 +3332,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3413,7 +3572,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -15716,7 +15874,6 @@
           <t>INT</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>INT0654</t>
@@ -15740,14 +15897,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -15758,27 +15919,968 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Perfil coluna</t>
+          <t>Código SA</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Comprimento (mm)</t>
+          <t>Cota A: centro a centro (mm)</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Código</t>
+          <t>Cota B: comprimento total (mm)</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
+          <t>Largura nominal da lateral (mm, pelo nome)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 0,18</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SA040287</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>72.93000000000001</v>
+      </c>
+      <c r="D2" t="n">
+        <v>103.43</v>
+      </c>
+      <c r="E2" t="n">
+        <v>180</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 0,30</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SA040183</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>189.72</v>
+      </c>
+      <c r="D3" t="n">
+        <v>220.22</v>
+      </c>
+      <c r="E3" t="n">
+        <v>300</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 0,55</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="n">
+        <v>443.7</v>
+      </c>
+      <c r="D4" t="n">
+        <v>474.2</v>
+      </c>
+      <c r="E4" t="n">
+        <v>550</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>SEM CÓDIGO</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>SA não cadastrado (SA**)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 0,60</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SA040318</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>490.9</v>
+      </c>
+      <c r="D5" t="n">
+        <v>521.4</v>
+      </c>
+      <c r="E5" t="n">
+        <v>600</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 0,70</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SA041218</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>590.9</v>
+      </c>
+      <c r="D6" t="n">
+        <v>621.4</v>
+      </c>
+      <c r="E6" t="n">
+        <v>700</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL LAT TRIPLA 0,74 MT – ESP</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SA041503</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>638.5</v>
+      </c>
+      <c r="D7" t="n">
+        <v>669</v>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL LAT TRIPLA 0,77 MT – ESP</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SA042003</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>663.5</v>
+      </c>
+      <c r="D8" t="n">
+        <v>694</v>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 0,80</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SA040269</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>690.9</v>
+      </c>
+      <c r="D9" t="n">
+        <v>721.4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>800</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 0,85</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SA040894</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>739.4</v>
+      </c>
+      <c r="D10" t="n">
+        <v>769.9</v>
+      </c>
+      <c r="E10" t="n">
+        <v>850</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 0,87</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SA040913</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>762.2</v>
+      </c>
+      <c r="D11" t="n">
+        <v>792.7</v>
+      </c>
+      <c r="E11" t="n">
+        <v>870</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 0,90</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>SA040206</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>790.9</v>
+      </c>
+      <c r="D12" t="n">
+        <v>821.4</v>
+      </c>
+      <c r="E12" t="n">
+        <v>900</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 0,95</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>SA041427</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>840.9</v>
+      </c>
+      <c r="D13" t="n">
+        <v>871.4</v>
+      </c>
+      <c r="E13" t="n">
+        <v>950</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 0,98</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SA041703</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>870.9</v>
+      </c>
+      <c r="D14" t="n">
+        <v>901.4</v>
+      </c>
+      <c r="E14" t="n">
+        <v>980</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 1,00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SA040004</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>890.9</v>
+      </c>
+      <c r="D15" t="n">
+        <v>921.4</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL LAT TRIPLA 2,00 MT - ESP</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SA040968</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>913.5</v>
+      </c>
+      <c r="D16" t="n">
+        <v>944</v>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 1,02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>SA041443</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>918.5</v>
+      </c>
+      <c r="D17" t="n">
+        <v>949</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>CONFERIR</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>A esperado 910.9 pela regra A−109,1: conferir</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 1,05</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>SA041705</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>940.9</v>
+      </c>
+      <c r="D18" t="n">
+        <v>971.4</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1050</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 1,07</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SA041299</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>962.5</v>
+      </c>
+      <c r="D19" t="n">
+        <v>993</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1070</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 1,10</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SA041029</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>999</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1029.5</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1100</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>CONFERIR</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>A esperado 990.9 pela regra A−109,1: conferir</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL LAT TRIPLA 2,21 MT - ESP</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>SA040926</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1017.5</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1048</v>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 1,20</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SA040911</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1090.9</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1121.4</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 1,25</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SA041027</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1143.5</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1174</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1250</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 1,30</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>SA041445</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1192.9</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1223.4</v>
+      </c>
+      <c r="E24" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 1,40</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SA041091</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1310</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1323.9</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1400</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>CONFERIR</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>B−A = 13.9 (esperado 30,5): conferir cadastro; A esperado 1290.9 pela regra A−109,1: conferir</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 1,42</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>SA041078</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1313.4</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1343.9</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1420</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL 1,60</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>SA040280</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1490.9</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1521.4</v>
+      </c>
+      <c r="E27" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL DRIVE IN 1,64</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SA041466</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1629.5</v>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL DRIVE IN 1,68</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>SA041467</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1643.9</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1674.4</v>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA HORIZONTAL DRIVE IN 1,89</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>SA041468</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1828.9</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1859.4</v>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E1"/>
+  <autoFilter ref="A1:H30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15789,14 +16891,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -15807,27 +16913,1255 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Perfil coluna</t>
+          <t>Código SA</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Comprimento (mm)</t>
+          <t>Cota A: centro a centro (mm)</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Código</t>
+          <t>Cota B: comprimento total (mm)</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
+          <t>Largura nominal da lateral (mm, pelo nome)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>V implícito (mm)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 0,18 - ESP LAT 3,00MT</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SA040286</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>456.29</v>
+      </c>
+      <c r="D2" t="n">
+        <v>486.79</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 0,18 X 0,55 - ESP TRAV</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SA040295</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>554.5</v>
+      </c>
+      <c r="D3" t="n">
+        <v>585</v>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 0,30</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SA040184</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>920.1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>950.6</v>
+      </c>
+      <c r="E4" t="n">
+        <v>300</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>900.1</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 0,80 - ESP 650 MM BAHAMAS</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SA041342</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>952</v>
+      </c>
+      <c r="D5" t="n">
+        <v>982.5</v>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL - ESP 2,60MT</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SA040222</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>957</v>
+      </c>
+      <c r="D6" t="n">
+        <v>987.5</v>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 0,85 - ESP 850 MM BAHAMAS</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SA041532</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>987.3000000000001</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1017.8</v>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 0,55</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="n">
+        <v>1003.3</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1033.8</v>
+      </c>
+      <c r="E8" t="n">
+        <v>550</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>901.2</v>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>SEM CÓDIGO</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>SA não cadastrado (SA**)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 0,60</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SA040317</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1026</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1056.5</v>
+      </c>
+      <c r="E9" t="n">
+        <v>600</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>900.9</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 0,80 ESP</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SA041288</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1057.38</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1087.88</v>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 1,00 ESP 1,08 MT</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SA040970</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1074</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1104.5</v>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 0,70</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>SA041217</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1077.38</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1107.88</v>
+      </c>
+      <c r="E12" t="n">
+        <v>700</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>900.9</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 1,02 ESP DREVIN</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>SA041666</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1097</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1127.5</v>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 1,00 - ESP 1000 MM BAHAMAS</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SA041533</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1102.8</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1133.3</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL LAT TRIPLA 0,74 MT – ESP</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SA041502</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1103.38</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1133.88</v>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL LAT TRIPLA 0,77 MT – ESP</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SA042002</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1118.38</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1148.88</v>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 0,80</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>SA040268</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1135</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1165.5</v>
+      </c>
+      <c r="E17" t="n">
+        <v>800</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>900.5</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 0,85</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>SA040893</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1165.2</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1195.7</v>
+      </c>
+      <c r="E18" t="n">
+        <v>850</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>899.3</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 0,87</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SA040912</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1179.8</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1210.3</v>
+      </c>
+      <c r="E19" t="n">
+        <v>870</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>901.6</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 0,90</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SA040205</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1198</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1228.5</v>
+      </c>
+      <c r="E20" t="n">
+        <v>900</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>899.8</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 0,95</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>SA041428</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1231.71</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1262.21</v>
+      </c>
+      <c r="E21" t="n">
+        <v>950</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>900</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 0,98</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SA041702</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1252.2</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1282.7</v>
+      </c>
+      <c r="E22" t="n">
+        <v>980</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>899.7</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 1,00</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SA040005</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1267</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1297.5</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>900.9</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL LAT TRIPLA 2,00 MT - ESP</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>SA040967</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1282.5</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1313</v>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 1,02</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SA041444</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1285.82</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1316.32</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>907.5</v>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>CONFERIR</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>V implícito fora de 600/900 (±3): conferir</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 1,05</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>SA041706</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1302</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1332.5</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1050</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>900</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 1,07</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>SA041304</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1318.82</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1349.32</v>
+      </c>
+      <c r="E27" t="n">
+        <v>1070</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>903.3</v>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>CONFERIR</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>V implícito fora de 600/900 (±3): conferir</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 1,00 ESP 1,36MT</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SA040305</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1333</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1363.5</v>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 1,10</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>SA041028</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1337.82</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1368.32</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1100</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>898.8</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL LAT TRIPLA 2,20 MT</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>SA041406</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1358.25</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1388.75</v>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 1,20</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>SA040910</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>1415.77</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1446.27</v>
+      </c>
+      <c r="E31" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>902.4</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 1,25</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>SA041026</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1455.1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>1485.6</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1250</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>903.1</v>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>CONFERIR</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>V implícito fora de 600/900 (±3): conferir</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 1,30</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>SA041446</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>1494.77</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1525.27</v>
+      </c>
+      <c r="E33" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>903.4</v>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>CONFERIR</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>V implícito fora de 600/900 (±3): conferir</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL LAT TRIPLA 1,40 MT - ESP</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>SA041077</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>1592.27</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1622.77</v>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 1,60</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>SA040279</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1741.5</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1772</v>
+      </c>
+      <c r="E35" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>padrão</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>900</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 2,74 ESP</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>SA042244</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>2740</v>
+      </c>
+      <c r="D36" t="n">
+        <v>2770.5</v>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA DIAGONAL 3,01 ESP</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>SA042245</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>3034</v>
+      </c>
+      <c r="D37" t="n">
+        <v>3064.5</v>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>especial/projeto</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E1"/>
+  <autoFilter ref="A1:I37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Exclude suspect horizontals, add code-format sheet, record travessa spacing rule
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0161y9YT6s3qhV5Y18zQkN9x
</commit_message>
<xml_diff>
--- a/drive-in/catalogo/CATALOGO.xlsx
+++ b/drive-in/catalogo/CATALOGO.xlsx
@@ -9,27 +9,28 @@
   <sheets>
     <sheet name="LEIA-ME" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Produtos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Composição" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Colunas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Sapatas" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Tala e fixadores" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Travessas" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Diagonais" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Placa niveladora" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Braços" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Outros" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Padrão de códigos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Composição" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Colunas" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Sapatas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Tala e fixadores" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Travessas" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Diagonais" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Placa niveladora" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Braços" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Outros" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Produtos'!$A$1:$S$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Composição'!$A$1:$G$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Colunas'!$A$1:$E$514</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sapatas'!$A$1:$G$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Tala e fixadores'!$A$1:$G$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Travessas'!$A$1:$H$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Diagonais'!$A$1:$I$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Placa niveladora'!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Braços'!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Outros'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Composição'!$A$1:$G$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Colunas'!$A$1:$E$514</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Sapatas'!$A$1:$G$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Tala e fixadores'!$A$1:$G$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Travessas'!$A$1:$H$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Diagonais'!$A$1:$I$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Placa niveladora'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Braços'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Outros'!$A$1:$E$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -55,7 +56,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -72,6 +73,11 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -85,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -96,6 +102,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -464,76 +471,72 @@
   <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="130" customWidth="1" min="1" max="1"/>
+    <col width="140" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CÓDIGOS DE ITENS – Drive-In</t>
+          <t>CATÁLOGO DE PRODUTOS – Drive-In</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>MESTRE DE DADOS: a aba "Produtos" concentra espessura, aço, dimensões, peso e quantidade de cada produto. O app lê SEMPRE daqui; nada é fixo no programa. Alterou uma célula, o cálculo muda.</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>"Peso usado no cálculo" é o valor que vale. "Peso do desenho (ref.)" é só comparação. Para mudar de fonte, edite a coluna "Peso usado".</t>
+          <t>MESTRE DE DADOS: a aba "Produtos" concentra aço, espessura, dimensões, peso e custo de cada produto. O app lê SEMPRE daqui; nada de produto é fixo no programa.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>"Custo unit. (R$)": preencher aqui (fixadores inclusive) para o app somar o custo.</t>
+          <t>"Peso usado no cálculo" é o valor que vale. "Peso do desenho (ref.)" é só comparação.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>"Composição": o que entra em cada conjunto (sapata, emenda) e em que quantidade. Parafusos e chumbadores ficam aqui, ligados ao item em "Produtos".</t>
+          <t>"Composição": o que entra em cada conjunto (sapata, emenda) e em que quantidade (parafusos e chumbadores inclusive).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Itens sem código entram no BOM como "SAXXXX" (regra do responsável técnico).</t>
+          <t>Abas por tipo de item (Colunas, Sapatas, Travessas, Diagonais...): só códigos e medidas. Em caso de dúvida ou erro, deixe o código em branco.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Travessas/Diagonais: o app procura o SA pelo comprimento calculado, tolerância ±3 mm.</t>
+          <t>Código em branco = item sem cadastro: o BOM usa o código provisório da aba "Padrão de códigos" (SA04XXXX, COXXXXXX, PAXXXXXX ou PKXXXXXX).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Em caso de dúvida ou erro, deixe o código em branco. Preencha depois; o app passa a usar assim que a aba for atualizada.</t>
+          <t>Travessas/Diagonais: o app procura o SA pelo comprimento calculado, tolerância de ±3 mm. Itens "EXCLUÍDO DA BUSCA" não são usados.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>A espessura NÃO faz parte do SA da coluna: o SA define só modelo + altura. A espessura é escolhida pelo usuário.</t>
+          <t>A espessura NÃO faz parte do SA da coluna: o SA define só modelo + altura.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Origem: tabelas de projeto 0004.0001.03.001/.003/.005, desenhos 0004.0001.03.007 (tala) e 0004.0003.02.001 (sapata).</t>
+          <t>Altura da estrutura: da parte inferior da sapata até o final do contraventamento superior (placa niveladora desprezada).</t>
         </is>
       </c>
     </row>
@@ -543,6 +546,120 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Prefixo</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Desenho</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Placa niveladora COL 80 e 101</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0004.0003.03.015</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>SA041463</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>mesma peça para 80 e 101</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Placa niveladora COL 122</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0004.0003.03.015</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SA041649</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -591,7 +708,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2841,7 +2958,6 @@
           <t>0004.0001.03.009</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
           <t>ACO0602 SLITER FF 1,40 x 80 GI</t>
@@ -2868,13 +2984,11 @@
           <t>calculado (sliter fechado)</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
           <t>por lateral (ver regras)</t>
         </is>
       </c>
-      <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2922,7 +3036,6 @@
           <t>0004.0001.03.009</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
           <t>ACO0602 SLITER FF 1,40 x 80 GI</t>
@@ -2949,13 +3062,11 @@
           <t>calculado (sliter fechado)</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
           <t>por vão entre horizontais</t>
         </is>
       </c>
-      <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2974,6 +3085,188 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Prefixo</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Formato no ERP</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Código provisório (sem cadastro)</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Significado</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Exemplo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SA000000 (as peças atuais são SA04xxxx)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SA04XXXX</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>semiacabado</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SA040045 (tala)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CO000000</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>COXXXXXX</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>composto / conjunto</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>CO040437 (sapata COL 101)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PA000000</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>PAXXXXXX</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>(a confirmar)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PK000000</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>PKXXXXXX</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>(a confirmar)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>INT0000 (fixadores)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>(a definir)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>fixadores / itens INT</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>INT0648 (parafuso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Regra: se o código da peça não existir no formato acima, o BOM usa o código provisório e entende-se que o item ainda não tem cadastro.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3894,7 +4187,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15430,7 +15723,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15725,7 +16018,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15891,7 +16184,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15983,7 +16276,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -16015,7 +16307,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -16023,7 +16314,6 @@
           <t>PP TRAVESSA HORIZONTAL 0,55</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
         <v>443.7</v>
       </c>
@@ -16079,7 +16369,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -16111,7 +16400,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -16130,7 +16418,6 @@
       <c r="D7" t="n">
         <v>669</v>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>especial/projeto</t>
@@ -16141,7 +16428,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -16160,7 +16446,6 @@
       <c r="D8" t="n">
         <v>694</v>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>especial/projeto</t>
@@ -16171,7 +16456,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -16203,7 +16487,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -16235,7 +16518,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -16267,7 +16549,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -16299,7 +16580,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -16331,7 +16611,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -16363,7 +16642,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -16395,7 +16673,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -16414,7 +16691,6 @@
       <c r="D16" t="n">
         <v>944</v>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>especial/projeto</t>
@@ -16425,39 +16701,38 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>PP TRAVESSA HORIZONTAL 1,02</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>SA041443</t>
         </is>
       </c>
-      <c r="C17" t="n">
+      <c r="C17" s="6" t="n">
         <v>918.5</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D17" s="6" t="n">
         <v>949</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="6" t="n">
         <v>1020</v>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>padrão</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>CONFERIR</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>EXCLUÍDO DA BUSCA</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>A esperado 910.9 pela regra A−109,1: conferir</t>
         </is>
@@ -16493,7 +16768,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -16525,39 +16799,38 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>PP TRAVESSA HORIZONTAL 1,10</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>SA041029</t>
         </is>
       </c>
-      <c r="C20" t="n">
+      <c r="C20" s="6" t="n">
         <v>999</v>
       </c>
-      <c r="D20" t="n">
+      <c r="D20" s="6" t="n">
         <v>1029.5</v>
       </c>
-      <c r="E20" t="n">
+      <c r="E20" s="6" t="n">
         <v>1100</v>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>padrão</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>CONFERIR</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>EXCLUÍDO DA BUSCA</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>A esperado 990.9 pela regra A−109,1: conferir</t>
         </is>
@@ -16580,7 +16853,6 @@
       <c r="D21" t="n">
         <v>1048</v>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>especial/projeto</t>
@@ -16591,7 +16863,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -16623,7 +16894,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -16655,7 +16925,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -16687,39 +16956,38 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>PP TRAVESSA HORIZONTAL 1,40</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>SA041091</t>
         </is>
       </c>
-      <c r="C25" t="n">
+      <c r="C25" s="6" t="n">
         <v>1310</v>
       </c>
-      <c r="D25" t="n">
+      <c r="D25" s="6" t="n">
         <v>1323.9</v>
       </c>
-      <c r="E25" t="n">
+      <c r="E25" s="6" t="n">
         <v>1400</v>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>padrão</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>CONFERIR</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>EXCLUÍDO DA BUSCA</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>B−A = 13.9 (esperado 30,5): conferir cadastro; A esperado 1290.9 pela regra A−109,1: conferir</t>
         </is>
@@ -16755,7 +17023,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -16787,7 +17054,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -16806,7 +17072,6 @@
       <c r="D28" t="n">
         <v>1629.5</v>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>especial/projeto</t>
@@ -16817,7 +17082,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -16836,7 +17100,6 @@
       <c r="D29" t="n">
         <v>1674.4</v>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>especial/projeto</t>
@@ -16847,7 +17110,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -16866,7 +17128,6 @@
       <c r="D30" t="n">
         <v>1859.4</v>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>especial/projeto</t>
@@ -16877,7 +17138,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H30"/>
@@ -16885,7 +17145,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -16969,19 +17229,16 @@
       <c r="D2" t="n">
         <v>486.79</v>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>especial/projeto</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -17000,19 +17257,16 @@
       <c r="D3" t="n">
         <v>585</v>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>especial/projeto</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -17047,7 +17301,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -17066,19 +17319,16 @@
       <c r="D5" t="n">
         <v>982.5</v>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>especial/projeto</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -17097,19 +17347,16 @@
       <c r="D6" t="n">
         <v>987.5</v>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>especial/projeto</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -17128,19 +17375,16 @@
       <c r="D7" t="n">
         <v>1017.8</v>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>especial/projeto</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -17148,7 +17392,6 @@
           <t>PP TRAVESSA DIAGONAL 0,55</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
         <v>1003.3</v>
       </c>
@@ -17210,7 +17453,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -17229,19 +17471,16 @@
       <c r="D10" t="n">
         <v>1087.88</v>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>especial/projeto</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -17260,19 +17499,16 @@
       <c r="D11" t="n">
         <v>1104.5</v>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>especial/projeto</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -17307,7 +17543,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -17326,19 +17561,16 @@
       <c r="D13" t="n">
         <v>1127.5</v>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>especial/projeto</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -17357,19 +17589,16 @@
       <c r="D14" t="n">
         <v>1133.3</v>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>especial/projeto</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -17388,19 +17617,16 @@
       <c r="D15" t="n">
         <v>1133.88</v>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>especial/projeto</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -17419,19 +17645,16 @@
       <c r="D16" t="n">
         <v>1148.88</v>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>especial/projeto</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -17466,7 +17689,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -17501,7 +17723,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -17536,7 +17757,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -17571,7 +17791,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -17606,7 +17825,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -17641,7 +17859,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -17676,7 +17893,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -17695,19 +17911,16 @@
       <c r="D24" t="n">
         <v>1313</v>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>especial/projeto</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -17781,7 +17994,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -17839,19 +18051,16 @@
       <c r="D28" t="n">
         <v>1363.5</v>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>especial/projeto</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -17886,7 +18095,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -17905,19 +18113,16 @@
       <c r="D30" t="n">
         <v>1388.75</v>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>especial/projeto</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -17952,7 +18157,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -18049,19 +18253,16 @@
       <c r="D34" t="n">
         <v>1622.77</v>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>especial/projeto</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -18096,7 +18297,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -18115,19 +18315,16 @@
       <c r="D36" t="n">
         <v>2770.5</v>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>especial/projeto</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -18146,136 +18343,19 @@
       <c r="D37" t="n">
         <v>3064.5</v>
       </c>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>especial/projeto</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Descrição</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>Prefixo</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>Desenho</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>Código</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>Observação</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Placa niveladora COL 80 e 101</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>SA</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>0004.0003.03.015</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>SA041463</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>mesma peça para 80 e 101</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Placa niveladora COL 122</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>SA</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>0004.0003.03.015</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>SA041649</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:E1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add horizontal travessa fasteners and tubo complemento rules
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0161y9YT6s3qhV5Y18zQkN9x
</commit_message>
<xml_diff>
--- a/drive-in/catalogo/CATALOGO.xlsx
+++ b/drive-in/catalogo/CATALOGO.xlsx
@@ -481,9 +481,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -714,7 +712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -748,6 +746,75 @@
       <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PP TUBO COMPLEMENTO TRAVESSA COL 80</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Tubo complemento</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>SA040047</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PP TUBO COMPLEMENTO TRAVESSA COL 101</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Tubo complemento</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SA040018</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PP TUBO COMPLEMENTO TRAVESSA COL 122</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Tubo complemento</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SA040046</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -763,7 +830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S33"/>
+  <dimension ref="A1:S38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3078,6 +3145,313 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>INT0993</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Fixador</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Parafuso sextavado 5/16" x 2.1/2" ZNC</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>INT0993</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>(sem peso)</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>ver Composição</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Travessa horizontal COL 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>INT0958</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Fixador</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Parafuso SX GR2 UNC R.P 5/16" x 3.1/4" zincado</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>INT0958</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>(sem peso)</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>ver Composição</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Travessa horizontal COL 101 (COL 122: a confirmar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>TUBO-80</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Tubo complemento</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>PP TUBO COMPLEMENTO TRAVESSA COL 80</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>80</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>SA040047</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M36" s="3" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>1 por nó sem diagonal</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Peso, aço e dimensões a informar</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>TUBO-101</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Tubo complemento</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>PP TUBO COMPLEMENTO TRAVESSA COL 101</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>101</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>SA040018</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M37" s="3" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>1 por nó sem diagonal</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>Peso, aço e dimensões a informar</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>TUBO-122</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Tubo complemento</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>PP TUBO COMPLEMENTO TRAVESSA COL 122</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>122</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>SA040046</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>1 por nó sem diagonal</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>Peso, aço e dimensões a informar</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:S30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3202,7 +3576,6 @@
           <t>(a confirmar)</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3225,7 +3598,6 @@
           <t>(a confirmar)</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3272,7 +3644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4178,6 +4550,309 @@
       <c r="G26" t="inlineStr">
         <is>
           <t>16 por tala</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TRAV-H (COL 80)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>INT0993</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Parafuso sextavado 5/16" x 2.1/2" ZNC</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>por travessa horizontal</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>1 em cada ponta</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>TRAV-H (COL 80)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>INT0650</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Porca sextavada 5/16" zincada</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>por travessa horizontal</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TRAV-H (COL 80)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>TUBO-80</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Tubo complemento travessa COL 80</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>por nó sem diagonal (máx. 2 por travessa)</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>nó com diagonal chegando NÃO usa tubo</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>TRAV-H (COL 101)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>INT0958</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Parafuso SX GR2 5/16" x 3.1/4" zinc.</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>por travessa horizontal</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>1 em cada ponta</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>TRAV-H (COL 101)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>INT0650</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Porca sextavada 5/16" zincada</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>por travessa horizontal</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>TRAV-H (COL 101)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>TUBO-101</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Tubo complemento travessa COL 101</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>por nó sem diagonal (máx. 2 por travessa)</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>nó com diagonal chegando NÃO usa tubo</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>TRAV-H (COL 122)</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>INT0958 ou INT0654</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Parafuso: código a confirmar</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>2</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>por travessa horizontal</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>A CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>a mensagem trazia 2 códigos (INT0958 e INT0654 chumbador)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>TRAV-H (COL 122)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>INT0650</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Porca sextavada 5/16" zincada</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>2</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>por travessa horizontal</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>TRAV-H (COL 122)</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>TUBO-122</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Tubo complemento travessa COL 122</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>por nó sem diagonal (máx. 2 por travessa)</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>nó com diagonal chegando NÃO usa tubo</t>
         </is>
       </c>
     </row>
@@ -16024,7 +16699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -16173,6 +16848,52 @@
         </is>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Parafuso sextavado 5/16" x 2.1/2" ZNC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>INT0993</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Parafuso SX GR2 UNC R.P 5/16" x 3.1/4" zincado</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>INT0958</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>OK</t>
         </is>

</xml_diff>

<commit_message>
Confirm horizontal travessa fasteners for COL 122 and tubo rule for all columns
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0161y9YT6s3qhV5Y18zQkN9x
</commit_message>
<xml_diff>
--- a/drive-in/catalogo/CATALOGO.xlsx
+++ b/drive-in/catalogo/CATALOGO.xlsx
@@ -481,7 +481,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -760,7 +759,6 @@
           <t>Tubo complemento</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>SA040047</t>
@@ -783,7 +781,6 @@
           <t>Tubo complemento</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>SA040018</t>
@@ -806,7 +803,6 @@
           <t>Tubo complemento</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>SA040046</t>
@@ -830,7 +826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S38"/>
+  <dimension ref="A1:S39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3176,29 +3172,21 @@
           <t>INT0993</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr">
         <is>
           <t>(sem peso)</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
           <t>ver Composição</t>
         </is>
       </c>
-      <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr">
         <is>
           <t>OK</t>
@@ -3241,29 +3229,21 @@
           <t>INT0958</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr">
         <is>
           <t>(sem peso)</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
           <t>ver Composição</t>
         </is>
       </c>
-      <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr">
         <is>
           <t>OK</t>
@@ -3271,7 +3251,7 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>Travessa horizontal COL 101 (COL 122: a confirmar)</t>
+          <t>Travessa horizontal COL 101</t>
         </is>
       </c>
     </row>
@@ -3304,25 +3284,17 @@
           <t>SA040047</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
       <c r="M36" s="3" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
-          <t>1 por nó sem diagonal</t>
-        </is>
-      </c>
-      <c r="Q36" t="inlineStr"/>
+          <t>2 por travessa horizontal, menos 1 por diagonal que chega (mín. 0)</t>
+        </is>
+      </c>
       <c r="R36" t="inlineStr">
         <is>
           <t>OK</t>
@@ -3363,25 +3335,17 @@
           <t>SA040018</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
       <c r="M37" s="3" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
-          <t>1 por nó sem diagonal</t>
-        </is>
-      </c>
-      <c r="Q37" t="inlineStr"/>
+          <t>2 por travessa horizontal, menos 1 por diagonal que chega (mín. 0)</t>
+        </is>
+      </c>
       <c r="R37" t="inlineStr">
         <is>
           <t>OK</t>
@@ -3422,25 +3386,17 @@
           <t>SA040046</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
       <c r="M38" s="3" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr">
         <is>
-          <t>1 por nó sem diagonal</t>
-        </is>
-      </c>
-      <c r="Q38" t="inlineStr"/>
+          <t>2 por travessa horizontal, menos 1 por diagonal que chega (mín. 0)</t>
+        </is>
+      </c>
       <c r="R38" t="inlineStr">
         <is>
           <t>OK</t>
@@ -3449,6 +3405,71 @@
       <c r="S38" t="inlineStr">
         <is>
           <t>Peso, aço e dimensões a informar</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>INT0973</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Fixador</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Parafuso sextavado 5/16" x 4" ZNC</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>122</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>INT0973</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>(sem peso)</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>ver Composição</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Travessa horizontal COL 122</t>
         </is>
       </c>
     </row>
@@ -4617,7 +4638,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4636,11 +4656,11 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>por nó sem diagonal (máx. 2 por travessa)</t>
+          <t>por travessa horizontal, menos 1 por diagonal que chega (mín. 0)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -4650,7 +4670,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>nó com diagonal chegando NÃO usa tubo</t>
+          <t>0, 1 ou 2 tubos por travessa; nó com diagonal não usa tubo (vale para COL 80, 101 e 122)</t>
         </is>
       </c>
     </row>
@@ -4718,7 +4738,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4737,11 +4756,11 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>por nó sem diagonal (máx. 2 por travessa)</t>
+          <t>por travessa horizontal, menos 1 por diagonal que chega (mín. 0)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -4751,7 +4770,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>nó com diagonal chegando NÃO usa tubo</t>
+          <t>0, 1 ou 2 tubos por travessa; nó com diagonal não usa tubo (vale para COL 80, 101 e 122)</t>
         </is>
       </c>
     </row>
@@ -4763,12 +4782,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>INT0958 ou INT0654</t>
+          <t>INT0973</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Parafuso: código a confirmar</t>
+          <t>Parafuso sextavado 5/16" x 4" ZNC</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -4779,14 +4798,14 @@
           <t>por travessa horizontal</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>A CONFIRMAR</t>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>a mensagem trazia 2 códigos (INT0958 e INT0654 chumbador)</t>
+          <t>1 em cada ponta</t>
         </is>
       </c>
     </row>
@@ -4819,7 +4838,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4838,11 +4856,11 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>por nó sem diagonal (máx. 2 por travessa)</t>
+          <t>por travessa horizontal, menos 1 por diagonal que chega (mín. 0)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4852,7 +4870,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>nó com diagonal chegando NÃO usa tubo</t>
+          <t>0, 1 ou 2 tubos por travessa; nó com diagonal não usa tubo (vale para COL 80, 101 e 122)</t>
         </is>
       </c>
     </row>
@@ -16699,7 +16717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -16864,7 +16882,6 @@
           <t>INT</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>INT0993</t>
@@ -16887,13 +16904,35 @@
           <t>INT</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>INT0958</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Parafuso sextavado 5/16" x 4" ZNC</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>INT0973</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>OK</t>
         </is>

</xml_diff>

<commit_message>
Add tubo complemento drawing data and diagonal fixing rule
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0161y9YT6s3qhV5Y18zQkN9x
</commit_message>
<xml_diff>
--- a/drive-in/catalogo/CATALOGO.xlsx
+++ b/drive-in/catalogo/CATALOGO.xlsx
@@ -734,7 +734,7 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Medida</t>
+          <t>Desenho</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
@@ -759,6 +759,11 @@
           <t>Tubo complemento</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0004.0001.03.010</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>SA040047</t>
@@ -781,6 +786,11 @@
           <t>Tubo complemento</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0004.0001.03.010</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>SA040018</t>
@@ -801,6 +811,11 @@
       <c r="B4" t="inlineStr">
         <is>
           <t>Tubo complemento</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0004.0001.03.010</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -3284,12 +3299,45 @@
           <t>SA040047</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>0004.0001.03.010</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>TUB0134 - TUBO REDONDO 1,2 x 1/2" x 6000</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Ø12,7 x 42</t>
+        </is>
+      </c>
       <c r="L36" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="M36" s="3" t="inlineStr"/>
+      <c r="M36" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>desenho</t>
+        </is>
+      </c>
+      <c r="O36" t="n">
+        <v>0.014</v>
+      </c>
       <c r="P36" t="inlineStr">
         <is>
           <t>2 por travessa horizontal, menos 1 por diagonal que chega (mín. 0)</t>
@@ -3300,11 +3348,7 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="S36" t="inlineStr">
-        <is>
-          <t>Peso, aço e dimensões a informar</t>
-        </is>
-      </c>
+      <c r="S36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3335,12 +3379,45 @@
           <t>SA040018</t>
         </is>
       </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>0004.0001.03.010</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>TUB0134 - TUBO REDONDO 1,2 x 1/2" x 6000</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Ø12,7 x 62</t>
+        </is>
+      </c>
       <c r="L37" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="M37" s="3" t="inlineStr"/>
+      <c r="M37" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>desenho</t>
+        </is>
+      </c>
+      <c r="O37" t="n">
+        <v>0.021</v>
+      </c>
       <c r="P37" t="inlineStr">
         <is>
           <t>2 por travessa horizontal, menos 1 por diagonal que chega (mín. 0)</t>
@@ -3351,11 +3428,7 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="S37" t="inlineStr">
-        <is>
-          <t>Peso, aço e dimensões a informar</t>
-        </is>
-      </c>
+      <c r="S37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3386,12 +3459,45 @@
           <t>SA040046</t>
         </is>
       </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>0004.0001.03.010</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>TUB0134 - TUBO REDONDO 1,2 x 1/2" x 6000</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Ø12,7 x 80</t>
+        </is>
+      </c>
       <c r="L38" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="M38" s="3" t="inlineStr"/>
+      <c r="M38" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>desenho</t>
+        </is>
+      </c>
+      <c r="O38" t="n">
+        <v>0.027</v>
+      </c>
       <c r="P38" t="inlineStr">
         <is>
           <t>2 por travessa horizontal, menos 1 por diagonal que chega (mín. 0)</t>
@@ -3402,11 +3508,7 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="S38" t="inlineStr">
-        <is>
-          <t>Peso, aço e dimensões a informar</t>
-        </is>
-      </c>
+      <c r="S38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3439,29 +3541,21 @@
           <t>INT0973</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr">
         <is>
           <t>(sem peso)</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr">
         <is>
           <t>ver Composição</t>
         </is>
       </c>
-      <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
           <t>OK</t>
@@ -16926,7 +17020,6 @@
           <t>INT</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>INT0973</t>

</xml_diff>

<commit_message>
Add travessa uniao (lateral tripla) variants from drawing
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0161y9YT6s3qhV5Y18zQkN9x
</commit_message>
<xml_diff>
--- a/drive-in/catalogo/CATALOGO.xlsx
+++ b/drive-in/catalogo/CATALOGO.xlsx
@@ -16,9 +16,10 @@
     <sheet name="Tala e fixadores" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Travessas" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Diagonais" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Placa niveladora" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Braços" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Outros" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Travessa união" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Placa niveladora" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Braços" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Outros" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Produtos'!$A$1:$S$30</definedName>
@@ -28,9 +29,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Tala e fixadores'!$A$1:$G$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Travessas'!$A$1:$H$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Diagonais'!$A$1:$I$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Placa niveladora'!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Braços'!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Outros'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Placa niveladora'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Braços'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Outros'!$A$1:$E$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -548,6 +549,392 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Coluna</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Código CO (conjunto)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Peso (kg, desenho)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>SA travessa montante triplo</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>SA perfil travamento posterior</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Cota interna (mm)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Comprimento total (mm)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Largura perfil posterior (mm)</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA UNIAO 1,05 LATERAL TRIPLA COL 80</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>80</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CO040165</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SA040925</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>SA040892</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>CONFERIR</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>cotas não constam no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA UNIAO 1,08 LATERAL TRIPLA COL 80</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>80</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CO040425</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1.493</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>SA041421</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>SA040892</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>CONFERIR</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>cotas não constam no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA UNIAO 0,70 LATERAL TRIPLA COL 80</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>80</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CO040458</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1.134</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SA041504</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>SA040892</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>664.7</v>
+      </c>
+      <c r="H4" t="n">
+        <v>696.5</v>
+      </c>
+      <c r="I4" t="n">
+        <v>84.59999999999999</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA UNIAO 1,03 LATERAL TRIPLA COL 101</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>101</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CO040356</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1.793</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>SA041303</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>SA040294</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>CONFERIR</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>cotas não constam no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA UNIAO 1,02 LATERAL TRIPLA COL 101</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>101</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CO040432</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1.793</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>SA041433</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>SA040294</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>986</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1017.8</v>
+      </c>
+      <c r="I6" t="n">
+        <v>106.6</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA UNIAO 0,76 LATERAL TRIPLA COL 101</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>101</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CO040755</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1.434</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>SA042089</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>SA040294</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>760</v>
+      </c>
+      <c r="H7" t="n">
+        <v>791.8</v>
+      </c>
+      <c r="I7" t="n">
+        <v>106.6</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA UNIAO 1,02 LATERAL TRIPLA COL 122</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>122</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CO040543</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2.059</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>SA041648</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>SA041647</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>986</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1017.8</v>
+      </c>
+      <c r="I8" t="n">
+        <v>126.6</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Fonte: desenho 0004.0001.02.011 REV.08. Conjunto soldado (GMAW): 1 travessa + 1 perfil de travamento posterior. Fixadores listados só na folha 0,70 COL 80: 6× INT0648 + 6× INT0650 (demais: a confirmar). Relação entre o comprimento e o passo A: a confirmar.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -656,7 +1043,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -705,7 +1092,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -841,7 +1228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S39"/>
+  <dimension ref="A1:S46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3348,7 +3735,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="S36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3428,7 +3814,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="S37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3508,7 +3893,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="S38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3564,6 +3948,575 @@
       <c r="S39" t="inlineStr">
         <is>
           <t>Travessa horizontal COL 122</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>UNIAO-80-1_05</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Travessa união</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA UNIAO 1,05 LATERAL TRIPLA COL 80</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>80</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>CO040165</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>0004.0001.02.011</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>(não especificado no desenho)</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M40" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>desenho</t>
+        </is>
+      </c>
+      <c r="O40" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>1 por nível de horizontal (coluna solteira)</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>conjunto soldado: SA040925 + SA040892</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>UNIAO-80-1_08</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Travessa união</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA UNIAO 1,08 LATERAL TRIPLA COL 80</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>80</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>CO040425</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>0004.0001.02.011</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>(não especificado no desenho)</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M41" t="n">
+        <v>1.493</v>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>desenho</t>
+        </is>
+      </c>
+      <c r="O41" t="n">
+        <v>1.493</v>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>1 por nível de horizontal (coluna solteira)</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>conjunto soldado: SA041421 + SA040892</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>UNIAO-80-0_70</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Travessa união</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA UNIAO 0,70 LATERAL TRIPLA COL 80</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>80</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>CO040458</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>0004.0001.02.011</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>(não especificado no desenho)</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>total 696.5</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M42" t="n">
+        <v>1.134</v>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>desenho</t>
+        </is>
+      </c>
+      <c r="O42" t="n">
+        <v>1.134</v>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>1 por nível de horizontal (coluna solteira)</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>conjunto soldado: SA041504 + SA040892</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>UNIAO-101-1_03</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Travessa união</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA UNIAO 1,03 LATERAL TRIPLA COL 101</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>101</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>CO040356</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>0004.0001.02.011</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>(não especificado no desenho)</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M43" t="n">
+        <v>1.793</v>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>desenho</t>
+        </is>
+      </c>
+      <c r="O43" t="n">
+        <v>1.793</v>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>1 por nível de horizontal (coluna solteira)</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>conjunto soldado: SA041303 + SA040294</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>UNIAO-101-1_02</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Travessa união</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA UNIAO 1,02 LATERAL TRIPLA COL 101</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>101</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>CO040432</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>0004.0001.02.011</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>(não especificado no desenho)</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>total 1017.8</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M44" t="n">
+        <v>1.793</v>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>desenho</t>
+        </is>
+      </c>
+      <c r="O44" t="n">
+        <v>1.793</v>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>1 por nível de horizontal (coluna solteira)</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>conjunto soldado: SA041433 + SA040294</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>UNIAO-101-0_76</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Travessa união</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA UNIAO 0,76 LATERAL TRIPLA COL 101</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>101</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>CO040755</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>0004.0001.02.011</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>(não especificado no desenho)</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>total 791.8</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M45" t="n">
+        <v>1.434</v>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>desenho</t>
+        </is>
+      </c>
+      <c r="O45" t="n">
+        <v>1.434</v>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>1 por nível de horizontal (coluna solteira)</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>conjunto soldado: SA042089 + SA040294</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>UNIAO-122-1_02</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Travessa união</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA UNIAO 1,02 LATERAL TRIPLA COL 122</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>122</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>CO040543</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>0004.0001.02.011</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>(não especificado no desenho)</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>total 1017.8</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M46" t="n">
+        <v>2.059</v>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>desenho</t>
+        </is>
+      </c>
+      <c r="O46" t="n">
+        <v>2.059</v>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>1 por nível de horizontal (coluna solteira)</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>conjunto soldado: SA041648 + SA041647</t>
         </is>
       </c>
     </row>
@@ -3759,7 +4712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4965,6 +5918,76 @@
       <c r="G35" t="inlineStr">
         <is>
           <t>0, 1 ou 2 tubos por travessa; nó com diagonal não usa tubo (vale para COL 80, 101 e 122)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>UNIAO (por peça)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>INT0648</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Parafuso 5/16" x 3/4" UNC ZNB</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>6</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>por travessa união</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>A CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>listado só na folha 0,70 COL 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>UNIAO (por peça)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>INT0650</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Porca sextavada 5/16" zincada</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>6</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>por travessa união</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>A CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>listado só na folha 0,70 COL 80</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Back beam uses top-beam profile (orange layer); top and back zig-zag diagonals only with 2 INT1193 + 2 INT0650 each; INT1193 added to catalog
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0161y9YT6s3qhV5Y18zQkN9x
</commit_message>
<xml_diff>
--- a/drive-in/catalogo/CATALOGO.xlsx
+++ b/drive-in/catalogo/CATALOGO.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="LEIA-ME" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Produtos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Padrão de códigos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Composição" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Colunas" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Sapatas" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Tala e fixadores" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Travessas" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Diagonais" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Travessa união" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Placa niveladora" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Braços" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Outros" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEIA-ME" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produtos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Padrão de códigos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Composição" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colunas" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sapatas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tala e fixadores" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Travessas" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagonais" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Travessa união" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Placa niveladora" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Braços" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outros" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Produtos'!$A$1:$S$30</definedName>
@@ -649,9 +649,6 @@
           <t>SA040892</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" s="3" t="inlineStr">
         <is>
           <t>CONFERIR</t>
@@ -690,9 +687,6 @@
           <t>SA040892</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" s="3" t="inlineStr">
         <is>
           <t>CONFERIR</t>
@@ -745,7 +739,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -774,9 +767,6 @@
           <t>SA040294</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" s="3" t="inlineStr">
         <is>
           <t>CONFERIR</t>
@@ -829,7 +819,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -872,7 +861,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -915,7 +903,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1228,7 +1215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S46"/>
+  <dimension ref="A1:S47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3954,71 +3941,44 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>UNIAO-80-1_05</t>
+          <t>INT1193</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Travessa união</t>
+          <t>Fixador</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>PP TRAVESSA UNIAO 1,05 LATERAL TRIPLA COL 80</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>80</v>
+          <t>Parafuso sextavado 5/16" x 1"</t>
+        </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>CO040165</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>0004.0001.02.011</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>08</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>(não especificado no desenho)</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
+          <t>INT1193</t>
+        </is>
+      </c>
       <c r="L40" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="M40" t="n">
-        <v>1.499</v>
-      </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>desenho</t>
-        </is>
-      </c>
-      <c r="O40" t="n">
-        <v>1.499</v>
+          <t>(sem peso)</t>
+        </is>
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>1 por nível de horizontal (coluna solteira)</t>
-        </is>
-      </c>
-      <c r="Q40" t="inlineStr"/>
+          <t>ver Composição</t>
+        </is>
+      </c>
       <c r="R40" t="inlineStr">
         <is>
           <t>OK</t>
@@ -4026,14 +3986,14 @@
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>conjunto soldado: SA040925 + SA040892</t>
+          <t>Diagonais do zig-zag de topo e de fundo (2 por diagonal)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>UNIAO-80-1_08</t>
+          <t>UNIAO-80-1_05</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4043,7 +4003,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>PP TRAVESSA UNIAO 1,08 LATERAL TRIPLA COL 80</t>
+          <t>PP TRAVESSA UNIAO 1,05 LATERAL TRIPLA COL 80</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -4056,7 +4016,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>CO040425</t>
+          <t>CO040165</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -4074,15 +4034,13 @@
           <t>(não especificado no desenho)</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
       <c r="M41" t="n">
-        <v>1.493</v>
+        <v>1.499</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
@@ -4090,14 +4048,13 @@
         </is>
       </c>
       <c r="O41" t="n">
-        <v>1.493</v>
+        <v>1.499</v>
       </c>
       <c r="P41" t="inlineStr">
         <is>
           <t>1 por nível de horizontal (coluna solteira)</t>
         </is>
       </c>
-      <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr">
         <is>
           <t>OK</t>
@@ -4105,14 +4062,14 @@
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>conjunto soldado: SA041421 + SA040892</t>
+          <t>conjunto soldado: SA040925 + SA040892</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>UNIAO-80-0_70</t>
+          <t>UNIAO-80-1_08</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4122,7 +4079,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>PP TRAVESSA UNIAO 0,70 LATERAL TRIPLA COL 80</t>
+          <t>PP TRAVESSA UNIAO 1,08 LATERAL TRIPLA COL 80</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -4135,7 +4092,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>CO040458</t>
+          <t>CO040425</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -4153,19 +4110,13 @@
           <t>(não especificado no desenho)</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>total 696.5</t>
-        </is>
-      </c>
       <c r="L42" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
       <c r="M42" t="n">
-        <v>1.134</v>
+        <v>1.493</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
@@ -4173,14 +4124,13 @@
         </is>
       </c>
       <c r="O42" t="n">
-        <v>1.134</v>
+        <v>1.493</v>
       </c>
       <c r="P42" t="inlineStr">
         <is>
           <t>1 por nível de horizontal (coluna solteira)</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr">
         <is>
           <t>OK</t>
@@ -4188,14 +4138,14 @@
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>conjunto soldado: SA041504 + SA040892</t>
+          <t>conjunto soldado: SA041421 + SA040892</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>UNIAO-101-1_03</t>
+          <t>UNIAO-80-0_70</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4205,11 +4155,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>PP TRAVESSA UNIAO 1,03 LATERAL TRIPLA COL 101</t>
+          <t>PP TRAVESSA UNIAO 0,70 LATERAL TRIPLA COL 80</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -4218,7 +4168,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>CO040356</t>
+          <t>CO040458</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4236,15 +4186,18 @@
           <t>(não especificado no desenho)</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>total 696.5</t>
+        </is>
+      </c>
       <c r="L43" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
       <c r="M43" t="n">
-        <v>1.793</v>
+        <v>1.134</v>
       </c>
       <c r="N43" t="inlineStr">
         <is>
@@ -4252,14 +4205,13 @@
         </is>
       </c>
       <c r="O43" t="n">
-        <v>1.793</v>
+        <v>1.134</v>
       </c>
       <c r="P43" t="inlineStr">
         <is>
           <t>1 por nível de horizontal (coluna solteira)</t>
         </is>
       </c>
-      <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
           <t>OK</t>
@@ -4267,14 +4219,14 @@
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>conjunto soldado: SA041303 + SA040294</t>
+          <t>conjunto soldado: SA041504 + SA040892</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>UNIAO-101-1_02</t>
+          <t>UNIAO-101-1_03</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -4284,7 +4236,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>PP TRAVESSA UNIAO 1,02 LATERAL TRIPLA COL 101</t>
+          <t>PP TRAVESSA UNIAO 1,03 LATERAL TRIPLA COL 101</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -4297,7 +4249,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>CO040432</t>
+          <t>CO040356</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -4313,12 +4265,6 @@
       <c r="I44" t="inlineStr">
         <is>
           <t>(não especificado no desenho)</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>total 1017.8</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -4342,7 +4288,6 @@
           <t>1 por nível de horizontal (coluna solteira)</t>
         </is>
       </c>
-      <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr">
         <is>
           <t>OK</t>
@@ -4350,14 +4295,14 @@
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>conjunto soldado: SA041433 + SA040294</t>
+          <t>conjunto soldado: SA041303 + SA040294</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>UNIAO-101-0_76</t>
+          <t>UNIAO-101-1_02</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4367,7 +4312,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>PP TRAVESSA UNIAO 0,76 LATERAL TRIPLA COL 101</t>
+          <t>PP TRAVESSA UNIAO 1,02 LATERAL TRIPLA COL 101</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -4380,7 +4325,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>CO040755</t>
+          <t>CO040432</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4398,10 +4343,9 @@
           <t>(não especificado no desenho)</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr">
         <is>
-          <t>total 791.8</t>
+          <t>total 1017.8</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -4410,7 +4354,7 @@
         </is>
       </c>
       <c r="M45" t="n">
-        <v>1.434</v>
+        <v>1.793</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
@@ -4418,14 +4362,13 @@
         </is>
       </c>
       <c r="O45" t="n">
-        <v>1.434</v>
+        <v>1.793</v>
       </c>
       <c r="P45" t="inlineStr">
         <is>
           <t>1 por nível de horizontal (coluna solteira)</t>
         </is>
       </c>
-      <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr">
         <is>
           <t>OK</t>
@@ -4433,88 +4376,167 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>conjunto soldado: SA042089 + SA040294</t>
+          <t>conjunto soldado: SA041433 + SA040294</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>UNIAO-101-0_76</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Travessa união</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>PP TRAVESSA UNIAO 0,76 LATERAL TRIPLA COL 101</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>101</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>CO040755</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>0004.0001.02.011</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>(não especificado no desenho)</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>total 791.8</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M46" t="n">
+        <v>1.434</v>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>desenho</t>
+        </is>
+      </c>
+      <c r="O46" t="n">
+        <v>1.434</v>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>1 por nível de horizontal (coluna solteira)</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>conjunto soldado: SA042089 + SA040294</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>UNIAO-122-1_02</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>Travessa união</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>PP TRAVESSA UNIAO 1,02 LATERAL TRIPLA COL 122</t>
         </is>
       </c>
-      <c r="D46" t="n">
+      <c r="D47" t="n">
         <v>122</v>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>CO</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>CO040543</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="G47" t="inlineStr">
         <is>
           <t>0004.0001.02.011</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="H47" t="inlineStr">
         <is>
           <t>08</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>(não especificado no desenho)</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr">
+      <c r="K47" t="inlineStr">
         <is>
           <t>total 1017.8</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
+      <c r="L47" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="M46" t="n">
+      <c r="M47" t="n">
         <v>2.059</v>
       </c>
-      <c r="N46" t="inlineStr">
+      <c r="N47" t="inlineStr">
         <is>
           <t>desenho</t>
         </is>
       </c>
-      <c r="O46" t="n">
+      <c r="O47" t="n">
         <v>2.059</v>
       </c>
-      <c r="P46" t="inlineStr">
+      <c r="P47" t="inlineStr">
         <is>
           <t>1 por nível de horizontal (coluna solteira)</t>
         </is>
       </c>
-      <c r="Q46" t="inlineStr"/>
-      <c r="R46" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="S46" t="inlineStr">
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
         <is>
           <t>conjunto soldado: SA041648 + SA041647</t>
         </is>

</xml_diff>

<commit_message>
Top/back beams from TB 80 models (PK codes and kit weights, linear fallback); project save/open as file with header; bend radius confirmed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0161y9YT6s3qhV5Y18zQkN9x
</commit_message>
<xml_diff>
--- a/drive-in/catalogo/CATALOGO.xlsx
+++ b/drive-in/catalogo/CATALOGO.xlsx
@@ -1215,7 +1215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S47"/>
+  <dimension ref="A1:S52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4539,6 +4539,321 @@
       <c r="S47" t="inlineStr">
         <is>
           <t>conjunto soldado: SA041648 + SA041647</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>LGTB80-1350</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Longarina TB 80 (topo/fundo)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>PP LONG 1,35 TB 80 - ESP DRIVE IN – kit com 2 INT0648 + 2 INT0650</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>PK041365</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>0004.0003.01.011</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>REV.05</t>
+        </is>
+      </c>
+      <c r="K48" t="n">
+        <v>1350</v>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M48" t="n">
+        <v>3.119</v>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>desenho (peso do kit)</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>conjunto CO041034; comprimento = largura nominal da rua</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>LGTB80-1400</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Longarina TB 80 (topo/fundo)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>PP LONG 1,40 TB 80 - ESP DRIVE IN – kit com 2 INT0648 + 2 INT0650</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>PK041334</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>0004.0003.01.011</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>REV.05</t>
+        </is>
+      </c>
+      <c r="K49" t="n">
+        <v>1400</v>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M49" t="n">
+        <v>3.215</v>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>desenho (peso do kit)</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>conjunto CO040447; comprimento = largura nominal da rua</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>LGTB80-1480</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Longarina TB 80 (topo/fundo)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>PP LONG 1,48 TB 80 - ESP DRIVE IN – kit com 2 INT0648 + 2 INT0650</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>PK041634</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>0004.0003.01.011</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>REV.05</t>
+        </is>
+      </c>
+      <c r="K50" t="n">
+        <v>1480</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M50" t="n">
+        <v>3.369</v>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>desenho (peso do kit)</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>conjunto CO041260; comprimento = largura nominal da rua</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>LGTB80-1570</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Longarina TB 80 (topo/fundo)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>PP LONG 1,57 TB 80 - ESP DRIVE IN – kit com 2 INT0648 + 2 INT0650</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>PK041446</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>0004.0003.01.011</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>REV.05</t>
+        </is>
+      </c>
+      <c r="K51" t="n">
+        <v>1570</v>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M51" t="n">
+        <v>3.541</v>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>desenho (peso do kit)</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>conjunto CO041092; comprimento = largura nominal da rua</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>LGTB80-1000T</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Longarina TB 80 (topo/fundo)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>PP LONG 1,00 TB 80 - ESP DRIVE IN TRAVAMENTO – kit com 2 INT0648 + 2 INT0650</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>PK041536</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>0004.0003.01.011</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>REV.05</t>
+        </is>
+      </c>
+      <c r="K52" t="n">
+        <v>996.3</v>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="M52" t="n">
+        <v>2.499</v>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>desenho (peso do kit)</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>conjunto CO041183; comprimento = largura nominal da rua</t>
         </is>
       </c>
     </row>

</xml_diff>